<commit_message>
Publish standalone digital acumen courses
</commit_message>
<xml_diff>
--- a/dla-course-2/downloads/SU_DLA_Solar_Completed_Reference_Workbook_V8.xlsx
+++ b/dla-course-2/downloads/SU_DLA_Solar_Completed_Reference_Workbook_V8.xlsx
@@ -1285,8 +1285,10 @@
       <x:c r="F39" s="115"/>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="8" t="str">
-        <x:v>Use Microsoft Excel or Google Sheets. Formulas, sheet names and course-critical cell addresses are identical; interface differences are explained on the Google Site.</x:v>
+      <x:c r="A40" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Complete the activity in Microsoft Excel. Google Sheets compatibility instructions are provided on the course site; sheet names and cell addresses remain the same.</x:t>
+        </x:is>
       </x:c>
       <x:c r="B40" s="8"/>
       <x:c r="C40" s="8"/>
@@ -2983,8 +2985,10 @@
       <x:c r="N2" s="41"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="43" t="str">
-        <x:v>The Production Manager challenges System C's 78% self-consumption assumption. Use the Google Site's supplied 20-year NPV formulas in B8:E8, then fill them down through row 14. Your task is to use and interrogate the discounted-cash-flow model, not build the full 20-year engine from first principles.</x:v>
+      <x:c r="A3" s="43" t="inlineStr">
+        <x:is>
+          <x:t>The first sensitivity row B8:E8 is supplied. Inspect the scenario reference $A8 in D8, then fill B8:E8 down through row 14. Refine the crossover by temporarily testing 74% and 73.9% in A14; restore 60% afterwards. Interpret the results rather than transcribing the NPV engine.</x:t>
+        </x:is>
       </x:c>
       <x:c r="B3" s="43"/>
       <x:c r="C3" s="43"/>
@@ -3457,8 +3461,10 @@
       <x:c r="N23" s="41"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="43" t="str">
-        <x:v>Use the Google Site formulas exactly as printed in either Excel or Google Sheets. SUMPRODUCT, ROW, MAX, MATCH, CHOOSE, absolute references and mixed references are used identically in this activity.</x:v>
+      <x:c r="A24" s="43" t="inlineStr">
+        <x:is>
+          <x:t>Microsoft Excel: use the fill handle to copy B8:E8 down to row 14. Google Sheets compatibility: select B8:E14 and use Fill down. The supplied NPV engine uses a fixed 20-year horizon and year-end cash flows.</x:t>
+        </x:is>
       </x:c>
       <x:c r="B24" s="43"/>
       <x:c r="C24" s="43"/>
@@ -4232,8 +4238,10 @@
       <x:c r="N28" s="41"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="102" t="str">
-        <x:v>Why can the shortest payback and the highest NPV point to different proposals?</x:v>
+      <x:c r="A29" s="102" t="inlineStr">
+        <x:is>
+          <x:t>Revisit: What did you initially think mattered most in choosing between the proposals?</x:t>
+        </x:is>
       </x:c>
       <x:c r="B29" s="102"/>
       <x:c r="C29" s="102"/>
@@ -4250,8 +4258,10 @@
       <x:c r="N29" s="41"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="102" t="str">
-        <x:v>Which assumption carries the highest financial risk in this case, and what evidence would you obtain?</x:v>
+      <x:c r="A30" s="102" t="inlineStr">
+        <x:is>
+          <x:t>Explain: Which result, assumption or sensitivity finding changed or strengthened your judgement, and why?</x:t>
+        </x:is>
       </x:c>
       <x:c r="B30" s="102"/>
       <x:c r="C30" s="102"/>
@@ -4268,8 +4278,10 @@
       <x:c r="N30" s="41"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="102" t="str">
-        <x:v>How does this modelling pattern transfer to another capital-allocation problem?</x:v>
+      <x:c r="A31" s="102" t="inlineStr">
+        <x:is>
+          <x:t>Transfer: Identify another business investment decision where this analytical pattern could be used.</x:t>
+        </x:is>
       </x:c>
       <x:c r="B31" s="102"/>
       <x:c r="C31" s="102"/>
@@ -4302,8 +4314,10 @@
       <x:c r="N32" s="41"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="102" t="str">
-        <x:v>Transfer pattern: Inputs → assumptions → calculation → alternatives → sensitivity → evidence → recommendation</x:v>
+      <x:c r="A33" s="102" t="inlineStr">
+        <x:is>
+          <x:t>Transfer pattern: Inputs → Model → Test assumptions → Interpret → Recommend</x:t>
+        </x:is>
       </x:c>
       <x:c r="B33" s="102"/>
       <x:c r="C33" s="102"/>

</xml_diff>